<commit_message>
Aggiunge nuovi bonus (Linea Impresa Efficiente, Conto Termico 3.0) al dossier Certosa
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Soluzioni_SI4.0_Certosa.xlsx
+++ b/Soluzioni_SI4.0_Certosa.xlsx
@@ -12,7 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Soluzioni" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chi sviluppa (make-or-buy)" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Allegato A - scaletta" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fonti" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nuovi bonus 28-09-2026" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approfondimento LIE + CT3.0" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fonti" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -101,6 +103,12 @@
       <sz val="9"/>
       <u val="single"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -140,7 +148,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -162,11 +170,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -251,6 +303,23 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -630,6 +699,7 @@
           <t>SI4.0 — Come partecipare</t>
         </is>
       </c>
+      <c r="B1" s="29" t="n"/>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -637,6 +707,7 @@
           <t>Bando SI4.0 2026 - Unioncamere Lombardia. Selezione a graduatoria (min 65/100). Agg. 17/09/2026: verificare sempre il testo ufficiale.</t>
         </is>
       </c>
+      <c r="B2" s="29" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -644,6 +715,7 @@
           <t>QUADRO GENERALE</t>
         </is>
       </c>
+      <c r="B3" s="29" t="n"/>
     </row>
     <row r="4" ht="59" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -723,6 +795,7 @@
           <t>REQUISITI ED ESCLUSIONI</t>
         </is>
       </c>
+      <c r="B10" s="29" t="n"/>
     </row>
     <row r="11" ht="44" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -754,6 +827,7 @@
           <t>TECNOLOGIE E SPESE</t>
         </is>
       </c>
+      <c r="B13" s="29" t="n"/>
     </row>
     <row r="14" ht="59" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
@@ -785,6 +859,7 @@
           <t>PROCEDURA</t>
         </is>
       </c>
+      <c r="B16" s="29" t="n"/>
     </row>
     <row r="17" ht="59" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
@@ -855,6 +930,7 @@
           <t>Certosa — fit e to—do</t>
         </is>
       </c>
+      <c r="B1" s="29" t="n"/>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -862,6 +938,7 @@
           <t>Certosa Servizi S.r.l. (Milano) - ESCO. Ammissibilita' e cose da fare entro il 25/09/2026.</t>
         </is>
       </c>
+      <c r="B2" s="29" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -869,6 +946,7 @@
           <t>AMMISSIBILITA'</t>
         </is>
       </c>
+      <c r="B3" s="29" t="n"/>
     </row>
     <row r="4" ht="29" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -912,6 +990,7 @@
           <t>IL NODO 'TELECONTROLLO'</t>
         </is>
       </c>
+      <c r="B7" s="29" t="n"/>
     </row>
     <row r="8" ht="59" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -931,6 +1010,7 @@
           <t>BLOCCA-O-PASSA (entro 25/09)</t>
         </is>
       </c>
+      <c r="B9" s="29" t="n"/>
     </row>
     <row r="10" ht="44" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
@@ -974,6 +1054,7 @@
           <t>COSA FARE OGGI</t>
         </is>
       </c>
+      <c r="B13" s="29" t="n"/>
     </row>
     <row r="14" ht="59" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
@@ -1028,6 +1109,15 @@
           <t>Soluzioni 4.0 sviluppabili da Certosa Servizi - Bando SI4.0 2026</t>
         </is>
       </c>
+      <c r="B1" s="30" t="n"/>
+      <c r="C1" s="30" t="n"/>
+      <c r="D1" s="30" t="n"/>
+      <c r="E1" s="30" t="n"/>
+      <c r="F1" s="30" t="n"/>
+      <c r="G1" s="30" t="n"/>
+      <c r="H1" s="30" t="n"/>
+      <c r="I1" s="30" t="n"/>
+      <c r="J1" s="29" t="n"/>
     </row>
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1035,6 +1125,15 @@
           <t>Il SI4.0 finanzia lo SVILUPPO di soluzioni nuove (non l'esistente). Il telecontrollo gia' in essere e' la BASE: la parte finanziabile e' il nuovo sviluppo sopra di esso. Priorita': le soluzioni che uniscono AI (+15) e impatto green misurabile (+15). Agg. 17/09/2026.</t>
         </is>
       </c>
+      <c r="B2" s="30" t="n"/>
+      <c r="C2" s="30" t="n"/>
+      <c r="D2" s="30" t="n"/>
+      <c r="E2" s="30" t="n"/>
+      <c r="F2" s="30" t="n"/>
+      <c r="G2" s="30" t="n"/>
+      <c r="H2" s="30" t="n"/>
+      <c r="I2" s="30" t="n"/>
+      <c r="J2" s="29" t="n"/>
     </row>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
@@ -1430,6 +1529,8 @@
           <t>Deve svilupparle Certosa o puo' pagare esterni?  (regole spese SI4.0 2026)</t>
         </is>
       </c>
+      <c r="B1" s="30" t="n"/>
+      <c r="C1" s="29" t="n"/>
     </row>
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="16" t="inlineStr">
@@ -1437,6 +1538,8 @@
           <t>Risposta breve: NON deve fare tutto in casa. Anzi il bando spinge sull'esterno (il personale interno conta solo fino al 30%). Attenzione a QUALI fornitori sono ammessi per ogni voce.</t>
         </is>
       </c>
+      <c r="B2" s="30" t="n"/>
+      <c r="C2" s="29" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
@@ -1563,6 +1666,8 @@
           <t>Vincoli sui fornitori (tutte le voci):</t>
         </is>
       </c>
+      <c r="B11" s="30" t="n"/>
+      <c r="C11" s="29" t="n"/>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
@@ -1570,6 +1675,8 @@
           <t>• Fornitori INDIPENDENTI: niente imprese collegate/controllate o infragruppo, niente conflitti di interesse.</t>
         </is>
       </c>
+      <c r="B12" s="30" t="n"/>
+      <c r="C12" s="29" t="n"/>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="9" t="inlineStr">
@@ -1577,6 +1684,8 @@
           <t>• Forniture a prezzi di mercato; PREVENTIVI obbligatori (da allegare).</t>
         </is>
       </c>
+      <c r="B13" s="30" t="n"/>
+      <c r="C13" s="29" t="n"/>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
@@ -1584,6 +1693,8 @@
           <t>• Spese ammissibili solo DALLA DATA DI APPROVAZIONE del bando (non l'esistente/gia' pagato).</t>
         </is>
       </c>
+      <c r="B14" s="30" t="n"/>
+      <c r="C14" s="29" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="9" t="inlineStr">
@@ -1591,6 +1702,8 @@
           <t>• Rendicontazione entro 12 mesi dalla concessione; fattura minima 300 EUR.</t>
         </is>
       </c>
+      <c r="B15" s="30" t="n"/>
+      <c r="C15" s="29" t="n"/>
     </row>
     <row r="17" ht="54" customHeight="1">
       <c r="A17" s="18" t="inlineStr">
@@ -1598,6 +1711,8 @@
           <t>IMPLICAZIONE PRATICA: conviene fare partnership con un DIH/EDIH/Competence Center/universita' per lo sviluppo AI: soddisfa il requisito 'fornitore qualificato' E porta il bonus +3 punti in graduatoria. Certosa coordina il progetto e mette il personale interno (entro il 30%).</t>
         </is>
       </c>
+      <c r="B17" s="30" t="n"/>
+      <c r="C17" s="29" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1634,6 +1749,7 @@
           <t>Allegato A 'Progetto' — scaletta e mappa punteggio</t>
         </is>
       </c>
+      <c r="B1" s="29" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1641,6 +1757,7 @@
           <t>Progetta ogni sezione per intercettare le voci di punteggio. (Il modello Word completo e' Scaletta_Allegato_A_SI4.0_Certosa.docx.)</t>
         </is>
       </c>
+      <c r="B2" s="29" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
@@ -1896,6 +2013,483 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>Nuovi bonus adatti a Certosa - aggiornato 28/09/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Chiusi di recente: SI4.0 2026 (25/9) e Impresa Sostenibile CCIAA Milano (3/9) -&gt; attendere ed. 2027. Restano aperti: Formazione Continua IV (31/3/2027), Rafforza &amp; Innova (31/3/2027), Competenze &amp; Innovazione (22/12/2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Bonus</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Ente</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Cosa da'</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Stato / scadenza</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Fonte</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="90" customHeight="1">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>Linea Impresa Efficiente ⭐</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Regione Lombardia (PR FESR / Finlombarda)</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Fondo perduto: fino a 45% su FER/cogenerazione; 20% micro-piccole / 15% medie su efficienza; 25% de minimis. + GARANZIA gratuita su finanziamento bancario fino 4,25 mln. Progetti 100k-5 mln EUR, riduzione emissioni &gt;=30%.</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>APERTO a sportello (dal 20/7/2026, fino a esaurimento)</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>ALTO</t>
+        </is>
+      </c>
+      <c r="F4" s="33" t="inlineStr">
+        <is>
+          <t>Apri</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="90" customHeight="1">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>Conto Termico 3.0 ⭐</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>GSE</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Incentivo su efficienza e rinnovabili termiche (pompe di calore, isolamento, nZEB, solare termico, FV se abbinato a PdC). Imprese: +20 p.p. piccole (fino ~65%), +10 p.p. medie. Una ESCO puo' fare da Soggetto Responsabile anche per conto terzi.</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>OPERATIVO (Portaltermico dal 2/2/2026), accesso diretto</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>ALTO</t>
+        </is>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>Apri</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="90" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Voucher Cloud e Cybersecurity</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>MIMIT (nazionale)</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>50% delle spese, max 20.000 EUR (min 4.000): software, servizi cloud e cybersecurity da fornitori accreditati MIMIT.</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Compilazione dal 20/10/2026; invio 10/11/2026 -&gt; 20/1/2027</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>ALTO</t>
+        </is>
+      </c>
+      <c r="F6" s="33" t="inlineStr">
+        <is>
+          <t>Apri</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="90" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>CER - tariffa incentivante</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>GSE</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Tariffa sull'energia condivisa (fino a 120 EUR/MWh). Il contributo a fondo perduto PNRR e' CHIUSO; resta la tariffa strutturale.</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>APERTA fino al 31/12/2027 (o esaurimento 5 GW)</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>Apri</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="90" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Nuova Sabatini</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>MIMIT (nazionale)</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Contributo su beni strumentali nuovi, inclusi beni digitali/4.0 (hardware/software).</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Sportello (fino a esaurimento)</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+      <c r="F8" s="33" t="inlineStr">
+        <is>
+          <t>Apri</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId5"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="94" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>Approfondimento: Linea Impresa Efficiente &amp; Conto Termico 3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="35" t="inlineStr">
+        <is>
+          <t>LINEA IMPRESA EFFICIENTE (Regione Lombardia)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Ente / gestione</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Regione Lombardia - PR FESR 2021-2027, Azione 2.1.3; attuazione Finlombarda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Obiettivo</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Efficientamento energetico dei processi produttivi (rinnovo dei sistemi produttivi + eventuale FER) per ridurre l'impatto ambientale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Beneficiari</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>PMI con sede operativa in Lombardia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Progetto</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Da 100.000 a 5.000.000 EUR; deve ridurre di almeno il 30% le emissioni climalteranti.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="54" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Contributo</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Fino a 45% su fonti rinnovabili/cogenerazione; efficienza energetica 20% micro-piccole, 15% medie; 25% in regime de minimis. In piu': garanzia gratuita regionale su finanziamento bancario fino a 4.250.000 EUR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Spese</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Fatture &gt; 1.000 EUR. ESCLUSE: leasing, usato, veicoli, opere edili, personale interno, formazione.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Cumulo</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Fino al 100% dei costi con altre agevolazioni; VIETATO il cumulo con PNRR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Procedura</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>A sportello (ordine cronologico), online su Bandi e Servizi; aperto dal 20/7/2026 fino a esaurimento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Per Certosa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Usarlo sui PROPRI impianti/processi: fotovoltaico, cogenerazione, macchinari ad alta efficienza. Attenzione: progetto minimo 100.000 EUR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="35" t="inlineStr">
+        <is>
+          <t>CONTO TERMICO 3.0 (GSE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Ente / portale</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>GSE - Portaltermico 3.0. Operativo dal 2/2/2026 (portale riaperto il 13/4/2026 dopo sospensione per numero domande).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Interventi (imprese, Titolo II)</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Sostituzione impianti termici con pompe di calore, solare termico, isolamento involucro, trasformazione nZEB; fotovoltaico solo se contestuale a pompe di calore elettriche.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Percentuali imprese</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Intensita' di aiuto maggiorata: +20 p.p. per le piccole imprese (fino a ~65%), +10 p.p. per le medie. Fotovoltaico: base 20% + 5/10/15% (efficienza / moduli UE).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="54" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Requisiti imprese</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Risparmio di energia primaria non rinnovabile &gt;=10% (&gt;=20% per multi-intervento); APE pre e post; audit energetico per interventi rilevanti (es. impianti &gt; 200 kW); valutazione preliminare dell'impresa prima dei lavori.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Ruolo ESCO</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Una ESCO certificata puo' operare come SOGGETTO RESPONSABILE, anche per conto terzi -&gt; per Certosa e' una leva commerciale, non solo un contributo sui propri edifici.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Domanda</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Accesso diretto (o prenotazione in certi casi); domanda entro 90 giorni dalla fine dei lavori via Portaltermico 3.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Per Certosa</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Doppio uso: sui propri edifici/impianti E come Soggetto Responsabile per i clienti (Comuni, aziende, condomini).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B7"/>
@@ -1911,6 +2505,7 @@
           <t>Fonti</t>
         </is>
       </c>
+      <c r="B1" s="29" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="20" t="inlineStr">

</xml_diff>

<commit_message>
Aggiunge Gap analysis sicurezza e esito NIS2 al dossier Certosa
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Soluzioni_SI4.0_Certosa.xlsx
+++ b/Soluzioni_SI4.0_Certosa.xlsx
@@ -13,7 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approfondimento LIE + CT3.0" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Piano formativo NIS2" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist NIS2" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fonti" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap analysis sicurezza" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fonti" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="24">
+  <fonts count="28">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -165,8 +166,32 @@
       <color rgb="009C6500"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009C6500"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -233,8 +258,13 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -315,11 +345,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -476,6 +550,44 @@
     </xf>
     <xf numFmtId="0" fontId="23" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2276,6 +2388,11 @@
           <t>Piano formativo NIS2 - Voucher Formazione Continua Lombardia (IV ed.)</t>
         </is>
       </c>
+      <c r="B1" s="55" t="n"/>
+      <c r="C1" s="55" t="n"/>
+      <c r="D1" s="55" t="n"/>
+      <c r="E1" s="55" t="n"/>
+      <c r="F1" s="56" t="n"/>
     </row>
     <row r="2" ht="46" customHeight="1" s="34">
       <c r="A2" s="37" t="inlineStr">
@@ -2283,6 +2400,11 @@
           <t>Copertura voucher per dimensione: fino a 9 dip. = 90% | 10-50 dip. = 70% | oltre 50 = 50%. Tetti: 2.000 EUR/persona/anno e 50.000 EUR/impresa/anno. I corsi devono essere nel Catalogo regionale (formazione.servizirl.it), area digitale/tecnico-specialistica. Importi qui sotto INDICATIVI, da adattare.</t>
         </is>
       </c>
+      <c r="B2" s="55" t="n"/>
+      <c r="C2" s="55" t="n"/>
+      <c r="D2" s="55" t="n"/>
+      <c r="E2" s="55" t="n"/>
+      <c r="F2" s="56" t="n"/>
     </row>
     <row r="3" ht="24" customHeight="1" s="34">
       <c r="A3" s="38" t="inlineStr">
@@ -2482,6 +2604,11 @@
           <t>Nota: verificare sul Catalogo regionale la presenza dei corsi cyber/NIS2/GDPR e l'ente accreditato che li eroga; rispettare i tetti per persona e per impresa.</t>
         </is>
       </c>
+      <c r="B11" s="55" t="n"/>
+      <c r="C11" s="55" t="n"/>
+      <c r="D11" s="55" t="n"/>
+      <c r="E11" s="55" t="n"/>
+      <c r="F11" s="56" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2500,7 +2627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="34" min="1" max="1"/>
@@ -2509,121 +2636,64 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" s="34">
-      <c r="A1" s="36" t="inlineStr">
+      <c r="A1" s="57" t="inlineStr">
         <is>
           <t>Checklist NIS2 - Certosa e' nel perimetro? Chi formare?</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="44" customHeight="1" s="34">
-      <c r="A2" s="37" t="inlineStr">
-        <is>
-          <t>NIS2 = Direttiva UE 2022/2555, in Italia D.Lgs. 138/2024. Non e' una 'certificazione': sono obblighi (registrazione ACN, misure di sicurezza, notifica incidenti, formazione, governance). Valutazione indicativa: la classificazione va confermata con ACN/consulente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1" s="34">
-      <c r="A3" s="49" t="inlineStr">
+    <row r="2" ht="22" customHeight="1" s="34">
+      <c r="A2" s="58" t="inlineStr">
+        <is>
+          <t>ESITO PER CERTOSA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="44" customHeight="1" s="34">
+      <c r="A3" s="39" t="inlineStr">
+        <is>
+          <t>Certosa NON e' (verosimilmente) soggetto NIS2 DIRETTO: non produce ne vende energia, 'vende gradi giorno' (Servizio Energia/gestione calore), non opera reti di teleriscaldamento. -&gt; Nessun obbligo di registrazione ACN come soggetto obbligato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1" s="34">
+      <c r="A4" s="59" t="inlineStr">
+        <is>
+          <t>DA CONFERMARE: che non gestiate una vera RETE di teleriscaldamento/teleraffrescamento (in tal caso, con dimensione media, potreste diventare 'importante').</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44" customHeight="1" s="34">
+      <c r="A5" s="39" t="inlineStr">
+        <is>
+          <t>MA esposizione via SUPPLY CHAIN: il telecontrollo da' accesso remoto agli impianti critici di Comuni/PA e ospedali (soggetti NIS2) -&gt; requisiti contrattuali di cybersecurity; siete fornitore ad alto rischio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1" s="34">
+      <c r="A6" s="39" t="inlineStr">
+        <is>
+          <t>PRIORITA': mettere in sicurezza il telecontrollo (vedi foglio 'Gap analysis sicurezza'). Finanziabile con Voucher Cloud/Cybersecurity + Formazione. Conformita' documentale = consulenza a parte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1" s="34">
+      <c r="A8" s="49" t="inlineStr">
         <is>
           <t>A) SEI NEL PERIMETRO NIS2?</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="50" t="inlineStr"/>
-      <c r="B4" s="46" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="50" t="inlineStr"/>
+      <c r="B9" s="46" t="inlineStr">
         <is>
           <t>Domanda</t>
         </is>
       </c>
-      <c r="C4" s="46" t="inlineStr">
+      <c r="C9" s="46" t="inlineStr">
         <is>
           <t>Se SI -&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1" s="34">
-      <c r="A5" s="51" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B5" s="52" t="inlineStr">
-        <is>
-          <t>Operate direttamente in un settore ad ALTA criticita' (All. I): energia elettrica/teleriscaldamento-raffrescamento/gas/idrogeno/oil, sanita', acqua, infrastrutture digitali, PA?</t>
-        </is>
-      </c>
-      <c r="C5" s="53" t="inlineStr">
-        <is>
-          <t>Possibile soggetto ESSENZIALE/IMPORTANTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1" s="34">
-      <c r="A6" s="51" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B6" s="52" t="inlineStr">
-        <is>
-          <t>Oppure in un settore critico (All. II): rifiuti, chimica, alimentare, MANIFATTURA (incl. dispositivi medici), fornitori digitali?</t>
-        </is>
-      </c>
-      <c r="C6" s="53" t="inlineStr">
-        <is>
-          <t>Possibile soggetto IMPORTANTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1" s="34">
-      <c r="A7" s="51" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B7" s="52" t="inlineStr">
-        <is>
-          <t>Dimensione: &gt;= 50 dipendenti OPPURE fatturato &gt; 10 mln EUR?</t>
-        </is>
-      </c>
-      <c r="C7" s="53" t="inlineStr">
-        <is>
-          <t>Soglia 'media impresa' -&gt; di norma NELL'ambito se settore elencato</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1" s="34">
-      <c r="A8" s="51" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B8" s="52" t="inlineStr">
-        <is>
-          <t>Dimensione: &gt;= 250 dipendenti OPPURE fatturato &gt; 50 mln EUR (e attivo &gt; 43 mln)?</t>
-        </is>
-      </c>
-      <c r="C8" s="53" t="inlineStr">
-        <is>
-          <t>Soglia 'grande' -&gt; tipicamente ESSENZIALE</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1" s="34">
-      <c r="A9" s="51" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B9" s="52" t="inlineStr">
-        <is>
-          <t>Fornite servizi a soggetti NIS2 (Comuni/PA, operatori energetici, ospedali)?</t>
-        </is>
-      </c>
-      <c r="C9" s="53" t="inlineStr">
-        <is>
-          <t>SUPPLY CHAIN: requisiti imposti dai clienti anche se non direttamente in ambito</t>
         </is>
       </c>
     </row>
@@ -2635,19 +2705,46 @@
       </c>
       <c r="B10" s="52" t="inlineStr">
         <is>
-          <t>Avete gia' verificato/effettuato la REGISTRAZIONE sul portale ACN?</t>
+          <t>Settore ad ALTA criticita' (All. I): energia elettrica/teleriscaldamento/gas/idrogeno/oil, sanita', acqua, infrastrutture digitali, PA?</t>
         </is>
       </c>
       <c r="C10" s="53" t="inlineStr">
         <is>
-          <t>Se no: verificare scadenze/calendario ACN 2026-2027</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1" s="34">
-      <c r="A12" s="49" t="inlineStr">
-        <is>
-          <t>B) FIGURE DA FORMARE (obbligo formativo NIS2)</t>
+          <t>Possibile ESSENZIALE/IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1" s="34">
+      <c r="A11" s="51" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B11" s="52" t="inlineStr">
+        <is>
+          <t>Settore critico (All. II): rifiuti, chimica, alimentare, MANIFATTURA (incl. dispositivi medici), fornitori digitali?</t>
+        </is>
+      </c>
+      <c r="C11" s="53" t="inlineStr">
+        <is>
+          <t>Possibile IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1" s="34">
+      <c r="A12" s="51" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B12" s="52" t="inlineStr">
+        <is>
+          <t>Dimensione: &gt;=50 dipendenti OPPURE fatturato &gt;10 mln EUR?</t>
+        </is>
+      </c>
+      <c r="C12" s="53" t="inlineStr">
+        <is>
+          <t>Soglia 'media' -&gt; nell'ambito se settore elencato</t>
         </is>
       </c>
     </row>
@@ -2659,12 +2756,12 @@
       </c>
       <c r="B13" s="52" t="inlineStr">
         <is>
-          <t>Organi di amministrazione / management (obbligo ESPLICITO NIS2)</t>
+          <t>Fornite servizi a soggetti NIS2 (Comuni/PA, operatori energetici, ospedali)?</t>
         </is>
       </c>
       <c r="C13" s="53" t="inlineStr">
         <is>
-          <t>Governance del rischio cyber</t>
+          <t>SUPPLY CHAIN -&gt; CASO DI CERTOSA</t>
         </is>
       </c>
     </row>
@@ -2676,46 +2773,19 @@
       </c>
       <c r="B14" s="52" t="inlineStr">
         <is>
-          <t>Responsabile sicurezza / IT manager</t>
+          <t>Registrazione sul portale ACN gia' verificata/effettuata?</t>
         </is>
       </c>
       <c r="C14" s="53" t="inlineStr">
         <is>
-          <t>Corso tecnico-gestionale</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1" s="34">
-      <c r="A15" s="51" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B15" s="52" t="inlineStr">
-        <is>
-          <t>Team IT/OT (sistemi di telecontrollo)</t>
-        </is>
-      </c>
-      <c r="C15" s="53" t="inlineStr">
-        <is>
-          <t>Sicurezza reti, gestione incidenti</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1" s="34">
-      <c r="A16" s="51" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B16" s="52" t="inlineStr">
-        <is>
-          <t>Tutti i dipendenti</t>
-        </is>
-      </c>
-      <c r="C16" s="53" t="inlineStr">
-        <is>
-          <t>Awareness cybersecurity</t>
+          <t>Se in ambito e non registrati: urgente</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1" s="34">
+      <c r="A16" s="49" t="inlineStr">
+        <is>
+          <t>B) FIGURE DA FORMARE</t>
         </is>
       </c>
     </row>
@@ -2727,19 +2797,46 @@
       </c>
       <c r="B17" s="52" t="inlineStr">
         <is>
-          <t>DPO / referente privacy</t>
+          <t>Organi di amministrazione / management (obbligo esplicito NIS2)</t>
         </is>
       </c>
       <c r="C17" s="53" t="inlineStr">
         <is>
-          <t>GDPR / protezione dati</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1" s="34">
-      <c r="A19" s="49" t="inlineStr">
-        <is>
-          <t>C) AZIONI PRIORITARIE</t>
+          <t>Governance rischio cyber</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1" s="34">
+      <c r="A18" s="51" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B18" s="52" t="inlineStr">
+        <is>
+          <t>Responsabile sicurezza / IT manager</t>
+        </is>
+      </c>
+      <c r="C18" s="53" t="inlineStr">
+        <is>
+          <t>Corso tecnico-gestionale</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1" s="34">
+      <c r="A19" s="51" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B19" s="52" t="inlineStr">
+        <is>
+          <t>Team IT/OT (telecontrollo)</t>
+        </is>
+      </c>
+      <c r="C19" s="53" t="inlineStr">
+        <is>
+          <t>Sicurezza reti, gestione incidenti</t>
         </is>
       </c>
     </row>
@@ -2751,10 +2848,14 @@
       </c>
       <c r="B20" s="52" t="inlineStr">
         <is>
-          <t>Verificare la classificazione (essenziale / importante / fuori ambito) e registrarsi su ACN</t>
-        </is>
-      </c>
-      <c r="C20" s="53" t="inlineStr"/>
+          <t>Tutti i dipendenti</t>
+        </is>
+      </c>
+      <c r="C20" s="53" t="inlineStr">
+        <is>
+          <t>Awareness cybersecurity</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1" s="34">
       <c r="A21" s="51" t="inlineStr">
@@ -2764,42 +2865,19 @@
       </c>
       <c r="B21" s="52" t="inlineStr">
         <is>
-          <t>Nominare referente e definire la governance del rischio</t>
-        </is>
-      </c>
-      <c r="C21" s="53" t="inlineStr"/>
-    </row>
-    <row r="22" ht="30" customHeight="1" s="34">
-      <c r="A22" s="51" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B22" s="52" t="inlineStr">
-        <is>
-          <t>Gap assessment delle misure di sicurezza vs requisiti NIS2</t>
-        </is>
-      </c>
-      <c r="C22" s="53" t="inlineStr">
-        <is>
-          <t>(consulenza - non coperta dai voucher)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1" s="34">
-      <c r="A23" s="51" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B23" s="52" t="inlineStr">
-        <is>
-          <t>Piano formativo -&gt; Voucher Formazione Continua Lombardia</t>
-        </is>
-      </c>
-      <c r="C23" s="53" t="inlineStr">
-        <is>
-          <t>(vedi foglio 'Piano formativo NIS2')</t>
+          <t>DPO / referente privacy</t>
+        </is>
+      </c>
+      <c r="C21" s="53" t="inlineStr">
+        <is>
+          <t>GDPR / protezione dati</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1" s="34">
+      <c r="A23" s="49" t="inlineStr">
+        <is>
+          <t>C) AZIONI PRIORITARIE</t>
         </is>
       </c>
     </row>
@@ -2811,29 +2889,93 @@
       </c>
       <c r="B24" s="52" t="inlineStr">
         <is>
-          <t>Implementazione misure tecniche -&gt; Voucher Cloud e Cybersecurity MIMIT</t>
-        </is>
-      </c>
-      <c r="C24" s="53" t="inlineStr">
-        <is>
-          <t>(firewall, EDR, backup, monitoraggio)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="28" customHeight="1" s="34">
-      <c r="A26" s="54" t="inlineStr">
-        <is>
-          <t>Disclaimer: valutazione orientativa. La qualifica NIS2 dipende da settore + dimensione e va confermata con ACN o un consulente specializzato.</t>
+          <t>Confermare con ACN/consulente la non-soggettivita' (verifica teleriscaldamento)</t>
+        </is>
+      </c>
+      <c r="C24" s="53" t="inlineStr"/>
+    </row>
+    <row r="25" ht="30" customHeight="1" s="34">
+      <c r="A25" s="51" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B25" s="52" t="inlineStr">
+        <is>
+          <t>Rispondere a questionari/clausole cyber dei clienti (supply chain)</t>
+        </is>
+      </c>
+      <c r="C25" s="53" t="inlineStr"/>
+    </row>
+    <row r="26" ht="30" customHeight="1" s="34">
+      <c r="A26" s="51" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B26" s="52" t="inlineStr">
+        <is>
+          <t>Mettere in sicurezza il TELECONTROLLO</t>
+        </is>
+      </c>
+      <c r="C26" s="53" t="inlineStr">
+        <is>
+          <t>-&gt; Voucher Cloud/Cybersecurity</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1" s="34">
+      <c r="A27" s="51" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B27" s="52" t="inlineStr">
+        <is>
+          <t>Piano formativo NIS2</t>
+        </is>
+      </c>
+      <c r="C27" s="53" t="inlineStr">
+        <is>
+          <t>-&gt; Voucher Formazione Continua</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1" s="34">
+      <c r="A28" s="51" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B28" s="52" t="inlineStr">
+        <is>
+          <t>Gap assessment / policy / governance</t>
+        </is>
+      </c>
+      <c r="C28" s="53" t="inlineStr">
+        <is>
+          <t>(consulenza - non coperta)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1" s="34">
+      <c r="A30" s="54" t="inlineStr">
+        <is>
+          <t>Disclaimer: valutazione orientativa, non parere legale. La qualifica NIS2 va confermata con ACN o un consulente.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A19:C19"/>
+  <mergeCells count="10">
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A6:C6"/>
     <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A4:C4"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2842,6 +2984,738 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" style="34" min="1" max="1"/>
+    <col width="22" customWidth="1" style="34" min="2" max="2"/>
+    <col width="10" customWidth="1" style="34" min="3" max="3"/>
+    <col width="20" customWidth="1" style="34" min="4" max="4"/>
+    <col width="42" customWidth="1" style="34" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1" s="34">
+      <c r="A1" s="57" t="inlineStr">
+        <is>
+          <t>Gap analysis sicurezza - Certosa (stato attuale vs cosa manca)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1" s="34">
+      <c r="A2" s="37" t="inlineStr">
+        <is>
+          <t>Base gia' presente: Firewall Cisco, MFA su account Microsoft, VPN accesso esterno, backup ogni 4h. Il Voucher Cloud/Cybersecurity finanzia SOLO il nuovo/migliorativo (non cio' che avete gia'). Verificare col fornitore le voci 'da verificare'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" s="34">
+      <c r="A3" s="38" t="inlineStr">
+        <is>
+          <t>Area / Misura</t>
+        </is>
+      </c>
+      <c r="B3" s="38" t="inlineStr">
+        <is>
+          <t>Stato</t>
+        </is>
+      </c>
+      <c r="C3" s="38" t="inlineStr">
+        <is>
+          <t>Prio.</t>
+        </is>
+      </c>
+      <c r="D3" s="38" t="inlineStr">
+        <is>
+          <t>Finanziabile Voucher</t>
+        </is>
+      </c>
+      <c r="E3" s="38" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" s="34">
+      <c r="A4" s="60" t="inlineStr">
+        <is>
+          <t>GIA' IN ESSERE (baseline - non finanziabile)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1" s="34">
+      <c r="A5" s="52" t="inlineStr">
+        <is>
+          <t>Firewall perimetrale (Cisco)</t>
+        </is>
+      </c>
+      <c r="B5" s="61" t="inlineStr">
+        <is>
+          <t>PRESENTE</t>
+        </is>
+      </c>
+      <c r="C5" s="62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D5" s="63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E5" s="52" t="inlineStr">
+        <is>
+          <t>Gia' in uso</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1" s="34">
+      <c r="A6" s="52" t="inlineStr">
+        <is>
+          <t>MFA su account Microsoft</t>
+        </is>
+      </c>
+      <c r="B6" s="61" t="inlineStr">
+        <is>
+          <t>PRESENTE</t>
+        </is>
+      </c>
+      <c r="C6" s="62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D6" s="63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E6" s="52" t="inlineStr">
+        <is>
+          <t>Estendere ad altri sistemi (vedi sotto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1" s="34">
+      <c r="A7" s="52" t="inlineStr">
+        <is>
+          <t>VPN per accesso esterno</t>
+        </is>
+      </c>
+      <c r="B7" s="61" t="inlineStr">
+        <is>
+          <t>PRESENTE</t>
+        </is>
+      </c>
+      <c r="C7" s="62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D7" s="63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E7" s="52" t="inlineStr">
+        <is>
+          <t>Valutare upgrade a ZTNA (nuovo = finanziabile)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1" s="34">
+      <c r="A8" s="52" t="inlineStr">
+        <is>
+          <t>Backup ogni 4 ore</t>
+        </is>
+      </c>
+      <c r="B8" s="61" t="inlineStr">
+        <is>
+          <t>PRESENTE</t>
+        </is>
+      </c>
+      <c r="C8" s="62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D8" s="63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E8" s="52" t="inlineStr">
+        <is>
+          <t>Verificare immutabilita'/DR (vedi sotto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" s="34">
+      <c r="A9" s="60" t="inlineStr">
+        <is>
+          <t>MANCA - PRIORITA' ALTA (soprattutto per il telecontrollo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1" s="34">
+      <c r="A10" s="52" t="inlineStr">
+        <is>
+          <t>Segmentazione rete OT/IT (DMZ telecontrollo)</t>
+        </is>
+      </c>
+      <c r="B10" s="64" t="inlineStr">
+        <is>
+          <t>MANCA</t>
+        </is>
+      </c>
+      <c r="C10" s="64" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="D10" s="63" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E10" s="52" t="inlineStr">
+        <is>
+          <t>Il firewall al perimetro non separa OT da office</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1" s="34">
+      <c r="A11" s="52" t="inlineStr">
+        <is>
+          <t>EDR/XDR su endpoint e server</t>
+        </is>
+      </c>
+      <c r="B11" s="65" t="inlineStr">
+        <is>
+          <t>DA VERIFICARE</t>
+        </is>
+      </c>
+      <c r="C11" s="64" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="D11" s="63" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E11" s="52" t="inlineStr">
+        <is>
+          <t>MFA+firewall non fermano ransomware; verificare col fornitore</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1" s="34">
+      <c r="A12" s="52" t="inlineStr">
+        <is>
+          <t>Monitoraggio/log + detection (SIEM/SOC 24/7)</t>
+        </is>
+      </c>
+      <c r="B12" s="65" t="inlineStr">
+        <is>
+          <t>DA VERIFICARE</t>
+        </is>
+      </c>
+      <c r="C12" s="64" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="D12" s="63" t="inlineStr">
+        <is>
+          <t>Si (serv. &lt;=30%)</t>
+        </is>
+      </c>
+      <c r="E12" s="52" t="inlineStr">
+        <is>
+          <t>Il fornitore fa detection o solo gestione?</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1" s="34">
+      <c r="A13" s="52" t="inlineStr">
+        <is>
+          <t>PAM + jump host per accessi al telecontrollo</t>
+        </is>
+      </c>
+      <c r="B13" s="64" t="inlineStr">
+        <is>
+          <t>MANCA</t>
+        </is>
+      </c>
+      <c r="C13" s="64" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="D13" s="63" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E13" s="52" t="inlineStr">
+        <is>
+          <t>Controllo/registrazione degli accessi privilegiati all'OT</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1" s="34">
+      <c r="A14" s="52" t="inlineStr">
+        <is>
+          <t>Backup immutabile/offline + test ripristino + DR</t>
+        </is>
+      </c>
+      <c r="B14" s="65" t="inlineStr">
+        <is>
+          <t>PARZIALE</t>
+        </is>
+      </c>
+      <c r="C14" s="64" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="D14" s="63" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E14" s="52" t="inlineStr">
+        <is>
+          <t>Avete la frequenza; serve resilienza al ransomware + DR</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1" s="34">
+      <c r="A15" s="60" t="inlineStr">
+        <is>
+          <t>MANCA - PRIORITA' MEDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1" s="34">
+      <c r="A16" s="52" t="inlineStr">
+        <is>
+          <t>Penetration test / Vulnerability Assessment periodico</t>
+        </is>
+      </c>
+      <c r="B16" s="64" t="inlineStr">
+        <is>
+          <t>MANCA</t>
+        </is>
+      </c>
+      <c r="C16" s="65" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="D16" s="63" t="inlineStr">
+        <is>
+          <t>Si (serv. &lt;=30%)</t>
+        </is>
+      </c>
+      <c r="E16" s="52" t="inlineStr">
+        <is>
+          <t>Gia' segnalato da voi</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1" s="34">
+      <c r="A17" s="52" t="inlineStr">
+        <is>
+          <t>Vulnerability &amp; patch management continuo (incl. OT)</t>
+        </is>
+      </c>
+      <c r="B17" s="64" t="inlineStr">
+        <is>
+          <t>MANCA</t>
+        </is>
+      </c>
+      <c r="C17" s="65" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="D17" s="63" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E17" s="52" t="inlineStr">
+        <is>
+          <t>Dispositivi OT spesso non aggiornati</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1" s="34">
+      <c r="A18" s="52" t="inlineStr">
+        <is>
+          <t>Cifratura dati e comunicazioni</t>
+        </is>
+      </c>
+      <c r="B18" s="65" t="inlineStr">
+        <is>
+          <t>DA VERIFICARE</t>
+        </is>
+      </c>
+      <c r="C18" s="65" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="D18" s="63" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E18" s="52" t="inlineStr">
+        <is>
+          <t>Telecontrollo + dati biomedicali/GDPR</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1" s="34">
+      <c r="A19" s="52" t="inlineStr">
+        <is>
+          <t>Email security avanzata / anti-phishing</t>
+        </is>
+      </c>
+      <c r="B19" s="65" t="inlineStr">
+        <is>
+          <t>DA VERIFICARE</t>
+        </is>
+      </c>
+      <c r="C19" s="65" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="D19" s="63" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E19" s="52" t="inlineStr">
+        <is>
+          <t>Phishing = vettore n.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1" s="34">
+      <c r="A20" s="52" t="inlineStr">
+        <is>
+          <t>MFA esteso (VPN, piattaforma telecontrollo, admin)</t>
+        </is>
+      </c>
+      <c r="B20" s="65" t="inlineStr">
+        <is>
+          <t>PARZIALE</t>
+        </is>
+      </c>
+      <c r="C20" s="65" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="D20" s="63" t="inlineStr">
+        <is>
+          <t>Si (nuove coperture)</t>
+        </is>
+      </c>
+      <c r="E20" s="52" t="inlineStr">
+        <is>
+          <t>Oggi solo account Microsoft</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1" s="34">
+      <c r="A21" s="60" t="inlineStr">
+        <is>
+          <t>ORGANIZZATIVE (consulenza - NON coperte dal voucher tecnologico)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1" s="34">
+      <c r="A22" s="52" t="inlineStr">
+        <is>
+          <t>Analisi del rischio + policy di sicurezza (ISO 27001)</t>
+        </is>
+      </c>
+      <c r="B22" s="64" t="inlineStr">
+        <is>
+          <t>MANCA</t>
+        </is>
+      </c>
+      <c r="C22" s="64" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="D22" s="63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E22" s="52" t="inlineStr">
+        <is>
+          <t>Consulenza</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1" s="34">
+      <c r="A23" s="52" t="inlineStr">
+        <is>
+          <t>Piano di risposta agli incidenti + notifica</t>
+        </is>
+      </c>
+      <c r="B23" s="64" t="inlineStr">
+        <is>
+          <t>MANCA</t>
+        </is>
+      </c>
+      <c r="C23" s="64" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="D23" s="63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E23" s="52" t="inlineStr">
+        <is>
+          <t>Consulenza / procedure</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1" s="34">
+      <c r="A24" s="52" t="inlineStr">
+        <is>
+          <t>Gestione supply chain (fornitori + requisiti clienti)</t>
+        </is>
+      </c>
+      <c r="B24" s="64" t="inlineStr">
+        <is>
+          <t>MANCA</t>
+        </is>
+      </c>
+      <c r="C24" s="65" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="D24" s="63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E24" s="52" t="inlineStr">
+        <is>
+          <t>Consulenza</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1" s="34">
+      <c r="A25" s="52" t="inlineStr">
+        <is>
+          <t>Inventario asset (soprattutto OT)</t>
+        </is>
+      </c>
+      <c r="B25" s="64" t="inlineStr">
+        <is>
+          <t>MANCA</t>
+        </is>
+      </c>
+      <c r="C25" s="65" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="D25" s="63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E25" s="52" t="inlineStr">
+        <is>
+          <t>Base per tutto il resto</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1" s="34">
+      <c r="A26" s="52" t="inlineStr">
+        <is>
+          <t>Formazione personale + management</t>
+        </is>
+      </c>
+      <c r="B26" s="64" t="inlineStr">
+        <is>
+          <t>MANCA</t>
+        </is>
+      </c>
+      <c r="C26" s="64" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="D26" s="63" t="inlineStr">
+        <is>
+          <t>Si (Formazione Continua)</t>
+        </is>
+      </c>
+      <c r="E26" s="52" t="inlineStr">
+        <is>
+          <t>Voucher diverso: Formazione Continua Lombardia</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1" s="34">
+      <c r="A28" s="66" t="inlineStr">
+        <is>
+          <t>PIANO DI SPESA VOUCHER SUI SOLI GAP (~40.000 EUR -&gt; contributo 20.000 EUR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1" s="34">
+      <c r="A29" s="41" t="inlineStr">
+        <is>
+          <t>EDR/XDR su endpoint e server</t>
+        </is>
+      </c>
+      <c r="E29" s="42" t="inlineStr">
+        <is>
+          <t>8.000 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1" s="34">
+      <c r="A30" s="39" t="inlineStr">
+        <is>
+          <t>SIEM + monitoraggio/SOC (servizio, &lt;=30%)</t>
+        </is>
+      </c>
+      <c r="E30" s="40" t="inlineStr">
+        <is>
+          <t>6.000 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1" s="34">
+      <c r="A31" s="41" t="inlineStr">
+        <is>
+          <t>Segmentazione rete OT/IT (apparati + configurazione)</t>
+        </is>
+      </c>
+      <c r="E31" s="42" t="inlineStr">
+        <is>
+          <t>8.000 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1" s="34">
+      <c r="A32" s="39" t="inlineStr">
+        <is>
+          <t>PAM / jump host per accessi al telecontrollo</t>
+        </is>
+      </c>
+      <c r="E32" s="40" t="inlineStr">
+        <is>
+          <t>7.000 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1" s="34">
+      <c r="A33" s="41" t="inlineStr">
+        <is>
+          <t>Backup immutabile + Disaster Recovery cloud</t>
+        </is>
+      </c>
+      <c r="E33" s="42" t="inlineStr">
+        <is>
+          <t>6.000 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1" s="34">
+      <c r="A34" s="39" t="inlineStr">
+        <is>
+          <t>Cifratura + email security avanzata</t>
+        </is>
+      </c>
+      <c r="E34" s="40" t="inlineStr">
+        <is>
+          <t>3.000 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1" s="34">
+      <c r="A35" s="41" t="inlineStr">
+        <is>
+          <t>Vulnerability assessment / penetration test (servizio, &lt;=30%)</t>
+        </is>
+      </c>
+      <c r="E35" s="42" t="inlineStr">
+        <is>
+          <t>2.000 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1" s="34">
+      <c r="A36" s="67" t="inlineStr">
+        <is>
+          <t>TOTALE PIANO -&gt; contributo 50% = 20.000 EUR</t>
+        </is>
+      </c>
+      <c r="E36" s="68" t="inlineStr">
+        <is>
+          <t>~40.000 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1" s="34">
+      <c r="A38" s="48" t="inlineStr">
+        <is>
+          <t>Nota: i servizi (SIEM 6k + VA/pen-test 2k = 8k) restano entro il 30% del piano. Importi indicativi, da adattare coi preventivi di un fornitore ACCREDITATO MIMIT. Ammesse solo soluzioni nuove/migliorative.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A36:D36"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>